<commit_message>
Fix app_view_selector warnings and implement active state retention
</commit_message>
<xml_diff>
--- a/example/Auto_Config.xlsx
+++ b/example/Auto_Config.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,16 +475,6 @@
           <t>field_8</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>field_9</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>field_10</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -513,108 +503,49 @@
       <c r="E5" t="n">
         <v>5</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>TestValue</t>
-        </is>
+      <c r="F5" t="n">
+        <v>2</v>
       </c>
       <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
         <v>2</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2010_qwerty</t>
+          <t>2020_qwerty</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20101</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>рынок
-цен
-за 
-такой-то год</t>
+          <t>20201</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>цены</t>
         </is>
       </c>
       <c r="E6" t="n">
+        <v>50</v>
+      </c>
+      <c r="F6" t="n">
+        <v>15</v>
+      </c>
+      <c r="G6" t="n">
         <v>5</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Хлеб</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
       <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2020_qwerty</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>20201</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>цены</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>50</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Хлеб</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>15</v>
-      </c>
-      <c r="H7" t="n">
         <v>5</v>
       </c>
-      <c r="I7" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refactor: Modularize project structure and clean up repo
</commit_message>
<xml_diff>
--- a/example/Auto_Config.xlsx
+++ b/example/Auto_Config.xlsx
@@ -423,7 +423,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>template_e.xlsx</t>
+          <t>../../../template_e.xlsx</t>
         </is>
       </c>
     </row>
@@ -482,15 +482,11 @@
           <t>2010_qwerty</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>20101</t>
-        </is>
+      <c r="B5" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C5" t="n">
+        <v>20101</v>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
@@ -519,15 +515,11 @@
           <t>2020_qwerty</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>20201</t>
-        </is>
+      <c r="B6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C6" t="n">
+        <v>20201</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>

</xml_diff>